<commit_message>
boolean value transformation, version bump, template update
</commit_message>
<xml_diff>
--- a/tests/fixtures/workbooks/a_workbook.xlsx
+++ b/tests/fixtures/workbooks/a_workbook.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10125"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/dev/ghga-transpiler/tests/fixtures/workbooks/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA669C62-E88B-9045-9712-220EAF6BA4EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E70CF1B1-C1D4-9144-BFCB-F7C1A1FAF516}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3300" yWindow="3740" windowWidth="42360" windowHeight="22280" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="12220" yWindow="9660" windowWidth="42360" windowHeight="22280" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="__properties" sheetId="16" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="23">
   <si>
     <t>writer_name</t>
   </si>
@@ -98,6 +98,12 @@
   </si>
   <si>
     <t>French Algeria</t>
+  </si>
+  <si>
+    <t>happy_ending</t>
+  </si>
+  <si>
+    <t>false</t>
   </si>
 </sst>
 </file>
@@ -380,7 +386,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{31EA5899-C9FA-1942-A6F2-92F5BCB75FA2}">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="16.1640625" customWidth="1"/>
@@ -389,7 +395,7 @@
     <col min="4" max="4" width="12.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -405,8 +411,11 @@
       <c r="E1" s="2" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="F1" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
@@ -422,8 +431,11 @@
       <c r="E2" s="2" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.15">
+      <c r="F2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.15">
       <c r="A3" s="2" t="s">
         <v>4</v>
       </c>
@@ -438,6 +450,9 @@
       </c>
       <c r="E3" s="2" t="s">
         <v>19</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>